<commit_message>
Updated ZAF_grids_kan model - 2025-12-11 11:10
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1994CFD9-6ACB-46E7-8DA2-706694FE59B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DA3452C-63A6-452D-9BA7-2C160A20D3FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -2549,7 +2549,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E0C4E1-EE9C-4292-AB5F-8E318D364D7E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FAB2CDE-2FCE-4498-A877-4E6C9A434FD4}">
   <dimension ref="B9:E237"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-25 09:17
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00AF8D48-C61C-46CE-AD08-83D6325D53AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{699F356B-95A9-4FB1-A13B-CEF80C3E49E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="574">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -349,1369 +349,1417 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_w62191005</t>
-  </si>
-  <si>
-    <t>e_w62191005*</t>
+    <t>p_w62191005-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w62191005-400_ZAF*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_w62193952</t>
-  </si>
-  <si>
-    <t>e_w62193952*</t>
-  </si>
-  <si>
-    <t>p_w62218063</t>
-  </si>
-  <si>
-    <t>e_w62218063*</t>
-  </si>
-  <si>
-    <t>p_w65600948</t>
-  </si>
-  <si>
-    <t>e_w65600948*</t>
-  </si>
-  <si>
-    <t>p_w75136015</t>
-  </si>
-  <si>
-    <t>e_w75136015*</t>
-  </si>
-  <si>
-    <t>p_w83525879</t>
-  </si>
-  <si>
-    <t>e_w83525879*</t>
-  </si>
-  <si>
-    <t>p_w87404898</t>
-  </si>
-  <si>
-    <t>e_w87404898*</t>
-  </si>
-  <si>
-    <t>p_w87434264</t>
-  </si>
-  <si>
-    <t>e_w87434264*</t>
-  </si>
-  <si>
-    <t>p_w89173873</t>
-  </si>
-  <si>
-    <t>e_w89173873*</t>
-  </si>
-  <si>
-    <t>p_w89637370</t>
-  </si>
-  <si>
-    <t>e_w89637370*</t>
-  </si>
-  <si>
-    <t>p_w90454383</t>
-  </si>
-  <si>
-    <t>e_w90454383*</t>
-  </si>
-  <si>
-    <t>p_w92348290</t>
-  </si>
-  <si>
-    <t>e_w92348290*</t>
-  </si>
-  <si>
-    <t>p_w98231311</t>
-  </si>
-  <si>
-    <t>e_w98231311*</t>
-  </si>
-  <si>
-    <t>p_w102682082</t>
-  </si>
-  <si>
-    <t>e_w102682082*</t>
-  </si>
-  <si>
-    <t>p_w102925909</t>
-  </si>
-  <si>
-    <t>e_w102925909*</t>
-  </si>
-  <si>
-    <t>p_w103079596</t>
-  </si>
-  <si>
-    <t>e_w103079596*</t>
-  </si>
-  <si>
-    <t>p_w104080393</t>
-  </si>
-  <si>
-    <t>e_w104080393*</t>
-  </si>
-  <si>
-    <t>p_w105759402</t>
-  </si>
-  <si>
-    <t>e_w105759402*</t>
-  </si>
-  <si>
-    <t>p_w105811523</t>
-  </si>
-  <si>
-    <t>e_w105811523*</t>
-  </si>
-  <si>
-    <t>p_w107391770</t>
-  </si>
-  <si>
-    <t>e_w107391770*</t>
-  </si>
-  <si>
-    <t>p_w107431792</t>
-  </si>
-  <si>
-    <t>e_w107431792*</t>
-  </si>
-  <si>
-    <t>p_w107937167</t>
-  </si>
-  <si>
-    <t>e_w107937167*</t>
-  </si>
-  <si>
-    <t>p_w120584910</t>
-  </si>
-  <si>
-    <t>e_w120584910*</t>
-  </si>
-  <si>
-    <t>p_w120941269</t>
-  </si>
-  <si>
-    <t>e_w120941269*</t>
-  </si>
-  <si>
-    <t>p_w125754107</t>
-  </si>
-  <si>
-    <t>e_w125754107*</t>
-  </si>
-  <si>
-    <t>p_w125769921</t>
-  </si>
-  <si>
-    <t>e_w125769921*</t>
-  </si>
-  <si>
-    <t>p_w127585817</t>
-  </si>
-  <si>
-    <t>e_w127585817*</t>
-  </si>
-  <si>
-    <t>p_w131625968</t>
-  </si>
-  <si>
-    <t>e_w131625968*</t>
-  </si>
-  <si>
-    <t>p_w142414070</t>
-  </si>
-  <si>
-    <t>e_w142414070*</t>
-  </si>
-  <si>
-    <t>p_w156418705</t>
-  </si>
-  <si>
-    <t>e_w156418705*</t>
-  </si>
-  <si>
-    <t>p_w162871098</t>
-  </si>
-  <si>
-    <t>e_w162871098*</t>
-  </si>
-  <si>
-    <t>p_w167540668</t>
-  </si>
-  <si>
-    <t>e_w167540668*</t>
-  </si>
-  <si>
-    <t>p_w167590549</t>
-  </si>
-  <si>
-    <t>e_w167590549*</t>
-  </si>
-  <si>
-    <t>p_w167648085</t>
-  </si>
-  <si>
-    <t>e_w167648085*</t>
-  </si>
-  <si>
-    <t>p_w169647963</t>
-  </si>
-  <si>
-    <t>e_w169647963*</t>
-  </si>
-  <si>
-    <t>p_w169789536</t>
-  </si>
-  <si>
-    <t>e_w169789536*</t>
-  </si>
-  <si>
-    <t>p_w170672051</t>
-  </si>
-  <si>
-    <t>e_w170672051*</t>
-  </si>
-  <si>
-    <t>p_w176362710</t>
-  </si>
-  <si>
-    <t>e_w176362710*</t>
-  </si>
-  <si>
-    <t>p_w176940672</t>
-  </si>
-  <si>
-    <t>e_w176940672*</t>
-  </si>
-  <si>
-    <t>p_w177800991</t>
-  </si>
-  <si>
-    <t>e_w177800991*</t>
-  </si>
-  <si>
-    <t>p_w178240552</t>
-  </si>
-  <si>
-    <t>e_w178240552*</t>
-  </si>
-  <si>
-    <t>p_w178968761</t>
-  </si>
-  <si>
-    <t>e_w178968761*</t>
-  </si>
-  <si>
-    <t>p_w179136373</t>
-  </si>
-  <si>
-    <t>e_w179136373*</t>
-  </si>
-  <si>
-    <t>p_w179140081</t>
-  </si>
-  <si>
-    <t>e_w179140081*</t>
-  </si>
-  <si>
-    <t>p_w181284049</t>
-  </si>
-  <si>
-    <t>e_w181284049*</t>
-  </si>
-  <si>
-    <t>p_w181366662</t>
-  </si>
-  <si>
-    <t>e_w181366662*</t>
-  </si>
-  <si>
-    <t>p_w182042518</t>
-  </si>
-  <si>
-    <t>e_w182042518*</t>
-  </si>
-  <si>
-    <t>p_w182408147</t>
-  </si>
-  <si>
-    <t>e_w182408147*</t>
-  </si>
-  <si>
-    <t>p_w183402339</t>
-  </si>
-  <si>
-    <t>e_w183402339*</t>
-  </si>
-  <si>
-    <t>p_w183757901</t>
-  </si>
-  <si>
-    <t>e_w183757901*</t>
-  </si>
-  <si>
-    <t>p_w183759046</t>
-  </si>
-  <si>
-    <t>e_w183759046*</t>
-  </si>
-  <si>
-    <t>p_w184201271</t>
-  </si>
-  <si>
-    <t>e_w184201271*</t>
-  </si>
-  <si>
-    <t>p_w184552955</t>
-  </si>
-  <si>
-    <t>e_w184552955*</t>
-  </si>
-  <si>
-    <t>p_w184560833</t>
-  </si>
-  <si>
-    <t>e_w184560833*</t>
-  </si>
-  <si>
-    <t>p_w184581460</t>
-  </si>
-  <si>
-    <t>e_w184581460*</t>
-  </si>
-  <si>
-    <t>p_w185171518</t>
-  </si>
-  <si>
-    <t>e_w185171518*</t>
-  </si>
-  <si>
-    <t>p_w185497473</t>
-  </si>
-  <si>
-    <t>e_w185497473*</t>
-  </si>
-  <si>
-    <t>p_w193465369</t>
-  </si>
-  <si>
-    <t>e_w193465369*</t>
-  </si>
-  <si>
-    <t>p_w193977981</t>
-  </si>
-  <si>
-    <t>e_w193977981*</t>
-  </si>
-  <si>
-    <t>p_w193978748</t>
-  </si>
-  <si>
-    <t>e_w193978748*</t>
-  </si>
-  <si>
-    <t>p_w200223220</t>
-  </si>
-  <si>
-    <t>e_w200223220*</t>
-  </si>
-  <si>
-    <t>p_w200232961</t>
-  </si>
-  <si>
-    <t>e_w200232961*</t>
-  </si>
-  <si>
-    <t>p_w200757306</t>
-  </si>
-  <si>
-    <t>e_w200757306*</t>
-  </si>
-  <si>
-    <t>p_w207991752</t>
-  </si>
-  <si>
-    <t>e_w207991752*</t>
-  </si>
-  <si>
-    <t>p_w208749745</t>
-  </si>
-  <si>
-    <t>e_w208749745*</t>
-  </si>
-  <si>
-    <t>p_w209365700</t>
-  </si>
-  <si>
-    <t>e_w209365700*</t>
-  </si>
-  <si>
-    <t>p_w209976655</t>
-  </si>
-  <si>
-    <t>e_w209976655*</t>
-  </si>
-  <si>
-    <t>p_w213181313</t>
-  </si>
-  <si>
-    <t>e_w213181313*</t>
-  </si>
-  <si>
-    <t>p_w219384657</t>
-  </si>
-  <si>
-    <t>e_w219384657*</t>
-  </si>
-  <si>
-    <t>p_w219596295</t>
-  </si>
-  <si>
-    <t>e_w219596295*</t>
-  </si>
-  <si>
-    <t>p_w220129604</t>
-  </si>
-  <si>
-    <t>e_w220129604*</t>
-  </si>
-  <si>
-    <t>p_w230551819</t>
-  </si>
-  <si>
-    <t>e_w230551819*</t>
-  </si>
-  <si>
-    <t>p_w238322344</t>
-  </si>
-  <si>
-    <t>e_w238322344*</t>
-  </si>
-  <si>
-    <t>p_w260486370</t>
-  </si>
-  <si>
-    <t>e_w260486370*</t>
-  </si>
-  <si>
-    <t>p_w359805008</t>
-  </si>
-  <si>
-    <t>e_w359805008*</t>
-  </si>
-  <si>
-    <t>p_w455498147</t>
-  </si>
-  <si>
-    <t>e_w455498147*</t>
-  </si>
-  <si>
-    <t>p_w496302277</t>
-  </si>
-  <si>
-    <t>e_w496302277*</t>
-  </si>
-  <si>
-    <t>p_w545652232</t>
-  </si>
-  <si>
-    <t>e_w545652232*</t>
-  </si>
-  <si>
-    <t>p_w586032034</t>
-  </si>
-  <si>
-    <t>e_w586032034*</t>
-  </si>
-  <si>
-    <t>p_w631673098</t>
-  </si>
-  <si>
-    <t>e_w631673098*</t>
-  </si>
-  <si>
-    <t>p_w663042845</t>
-  </si>
-  <si>
-    <t>e_w663042845*</t>
-  </si>
-  <si>
-    <t>p_w663042849</t>
-  </si>
-  <si>
-    <t>e_w663042849*</t>
-  </si>
-  <si>
-    <t>p_w685294883</t>
-  </si>
-  <si>
-    <t>e_w685294883*</t>
-  </si>
-  <si>
-    <t>p_w693869805</t>
-  </si>
-  <si>
-    <t>e_w693869805*</t>
-  </si>
-  <si>
-    <t>p_w836844162</t>
-  </si>
-  <si>
-    <t>e_w836844162*</t>
-  </si>
-  <si>
-    <t>p_w934819484</t>
-  </si>
-  <si>
-    <t>e_w934819484*</t>
-  </si>
-  <si>
-    <t>p_w1146812331</t>
-  </si>
-  <si>
-    <t>e_w1146812331*</t>
-  </si>
-  <si>
-    <t>p_w1146878078</t>
-  </si>
-  <si>
-    <t>e_w1146878078*</t>
-  </si>
-  <si>
-    <t>p_r17287657</t>
-  </si>
-  <si>
-    <t>e_r17287657*</t>
-  </si>
-  <si>
-    <t>p_ZA25</t>
-  </si>
-  <si>
-    <t>e_ZA25*</t>
-  </si>
-  <si>
-    <t>p_ZA20</t>
-  </si>
-  <si>
-    <t>e_ZA20*</t>
-  </si>
-  <si>
-    <t>p_ZA22</t>
-  </si>
-  <si>
-    <t>e_ZA22*</t>
-  </si>
-  <si>
-    <t>p_ZA29</t>
-  </si>
-  <si>
-    <t>e_ZA29*</t>
-  </si>
-  <si>
-    <t>p_ZA3</t>
-  </si>
-  <si>
-    <t>e_ZA3*</t>
-  </si>
-  <si>
-    <t>p_ZA23</t>
-  </si>
-  <si>
-    <t>e_ZA23*</t>
-  </si>
-  <si>
-    <t>p_ZA30</t>
-  </si>
-  <si>
-    <t>e_ZA30*</t>
-  </si>
-  <si>
-    <t>p_ZA18</t>
-  </si>
-  <si>
-    <t>e_ZA18*</t>
-  </si>
-  <si>
-    <t>p_ZA11</t>
-  </si>
-  <si>
-    <t>e_ZA11*</t>
-  </si>
-  <si>
-    <t>p_ZA40</t>
-  </si>
-  <si>
-    <t>e_ZA40*</t>
-  </si>
-  <si>
-    <t>p_ZA39</t>
-  </si>
-  <si>
-    <t>e_ZA39*</t>
-  </si>
-  <si>
-    <t>p_ZA26</t>
-  </si>
-  <si>
-    <t>e_ZA26*</t>
-  </si>
-  <si>
-    <t>p_ZA2</t>
-  </si>
-  <si>
-    <t>e_ZA2*</t>
-  </si>
-  <si>
-    <t>p_ZA7</t>
-  </si>
-  <si>
-    <t>e_ZA7*</t>
-  </si>
-  <si>
-    <t>p_ZA5</t>
-  </si>
-  <si>
-    <t>e_ZA5*</t>
-  </si>
-  <si>
-    <t>p_ZA6</t>
-  </si>
-  <si>
-    <t>e_ZA6*</t>
-  </si>
-  <si>
-    <t>p_ZA31</t>
-  </si>
-  <si>
-    <t>e_ZA31*</t>
-  </si>
-  <si>
-    <t>p_ZA15</t>
-  </si>
-  <si>
-    <t>e_ZA15*</t>
-  </si>
-  <si>
-    <t>p_ZA1</t>
-  </si>
-  <si>
-    <t>e_ZA1*</t>
-  </si>
-  <si>
-    <t>p_ZA36</t>
-  </si>
-  <si>
-    <t>e_ZA36*</t>
-  </si>
-  <si>
-    <t>p_ZA19</t>
-  </si>
-  <si>
-    <t>e_ZA19*</t>
-  </si>
-  <si>
-    <t>p_ZA24</t>
-  </si>
-  <si>
-    <t>e_ZA24*</t>
-  </si>
-  <si>
-    <t>p_ZA14</t>
-  </si>
-  <si>
-    <t>e_ZA14*</t>
-  </si>
-  <si>
-    <t>p_ZA17</t>
-  </si>
-  <si>
-    <t>e_ZA17*</t>
-  </si>
-  <si>
-    <t>p_ZA38</t>
-  </si>
-  <si>
-    <t>e_ZA38*</t>
-  </si>
-  <si>
-    <t>p_ZA16</t>
-  </si>
-  <si>
-    <t>e_ZA16*</t>
-  </si>
-  <si>
-    <t>p_ZA28</t>
-  </si>
-  <si>
-    <t>e_ZA28*</t>
-  </si>
-  <si>
-    <t>p_ZA4</t>
-  </si>
-  <si>
-    <t>e_ZA4*</t>
-  </si>
-  <si>
-    <t>p_ZA33</t>
-  </si>
-  <si>
-    <t>e_ZA33*</t>
-  </si>
-  <si>
-    <t>p_ZA42</t>
-  </si>
-  <si>
-    <t>e_ZA42*</t>
-  </si>
-  <si>
-    <t>p_ZA41</t>
-  </si>
-  <si>
-    <t>e_ZA41*</t>
-  </si>
-  <si>
-    <t>p_ZA43</t>
-  </si>
-  <si>
-    <t>e_ZA43*</t>
-  </si>
-  <si>
-    <t>p_ZA44</t>
-  </si>
-  <si>
-    <t>e_ZA44*</t>
-  </si>
-  <si>
-    <t>rez_spv_001</t>
-  </si>
-  <si>
-    <t>elc_spv_001</t>
-  </si>
-  <si>
-    <t>rez_spv_002</t>
-  </si>
-  <si>
-    <t>elc_spv_002</t>
-  </si>
-  <si>
-    <t>rez_spv_003</t>
-  </si>
-  <si>
-    <t>elc_spv_003</t>
-  </si>
-  <si>
-    <t>rez_spv_004</t>
-  </si>
-  <si>
-    <t>elc_spv_004</t>
-  </si>
-  <si>
-    <t>rez_spv_005</t>
-  </si>
-  <si>
-    <t>elc_spv_005</t>
-  </si>
-  <si>
-    <t>rez_spv_006</t>
-  </si>
-  <si>
-    <t>elc_spv_006</t>
-  </si>
-  <si>
-    <t>rez_spv_007</t>
-  </si>
-  <si>
-    <t>elc_spv_007</t>
-  </si>
-  <si>
-    <t>rez_spv_008</t>
-  </si>
-  <si>
-    <t>elc_spv_008</t>
-  </si>
-  <si>
-    <t>rez_spv_009</t>
-  </si>
-  <si>
-    <t>elc_spv_009</t>
-  </si>
-  <si>
-    <t>rez_spv_010</t>
-  </si>
-  <si>
-    <t>elc_spv_010</t>
-  </si>
-  <si>
-    <t>rez_spv_011</t>
-  </si>
-  <si>
-    <t>elc_spv_011</t>
-  </si>
-  <si>
-    <t>rez_spv_012</t>
-  </si>
-  <si>
-    <t>elc_spv_012</t>
-  </si>
-  <si>
-    <t>rez_spv_013</t>
-  </si>
-  <si>
-    <t>elc_spv_013</t>
-  </si>
-  <si>
-    <t>rez_spv_014</t>
-  </si>
-  <si>
-    <t>elc_spv_014</t>
-  </si>
-  <si>
-    <t>rez_spv_015</t>
-  </si>
-  <si>
-    <t>elc_spv_015</t>
-  </si>
-  <si>
-    <t>rez_spv_016</t>
-  </si>
-  <si>
-    <t>elc_spv_016</t>
-  </si>
-  <si>
-    <t>rez_spv_017</t>
-  </si>
-  <si>
-    <t>elc_spv_017</t>
-  </si>
-  <si>
-    <t>rez_spv_018</t>
-  </si>
-  <si>
-    <t>elc_spv_018</t>
-  </si>
-  <si>
-    <t>rez_spv_019</t>
-  </si>
-  <si>
-    <t>elc_spv_019</t>
-  </si>
-  <si>
-    <t>rez_spv_020</t>
-  </si>
-  <si>
-    <t>elc_spv_020</t>
-  </si>
-  <si>
-    <t>rez_spv_021</t>
-  </si>
-  <si>
-    <t>elc_spv_021</t>
-  </si>
-  <si>
-    <t>rez_spv_022</t>
-  </si>
-  <si>
-    <t>elc_spv_022</t>
-  </si>
-  <si>
-    <t>rez_spv_023</t>
-  </si>
-  <si>
-    <t>elc_spv_023</t>
-  </si>
-  <si>
-    <t>rez_spv_024</t>
-  </si>
-  <si>
-    <t>elc_spv_024</t>
-  </si>
-  <si>
-    <t>rez_spv_025</t>
-  </si>
-  <si>
-    <t>elc_spv_025</t>
-  </si>
-  <si>
-    <t>rez_spv_026</t>
-  </si>
-  <si>
-    <t>elc_spv_026</t>
-  </si>
-  <si>
-    <t>rez_spv_027</t>
-  </si>
-  <si>
-    <t>elc_spv_027</t>
-  </si>
-  <si>
-    <t>rez_spv_028</t>
-  </si>
-  <si>
-    <t>elc_spv_028</t>
-  </si>
-  <si>
-    <t>rez_spv_029</t>
-  </si>
-  <si>
-    <t>elc_spv_029</t>
-  </si>
-  <si>
-    <t>rez_spv_030</t>
-  </si>
-  <si>
-    <t>elc_spv_030</t>
-  </si>
-  <si>
-    <t>rez_spv_031</t>
-  </si>
-  <si>
-    <t>elc_spv_031</t>
-  </si>
-  <si>
-    <t>rez_spv_032</t>
-  </si>
-  <si>
-    <t>elc_spv_032</t>
-  </si>
-  <si>
-    <t>rez_spv_033</t>
-  </si>
-  <si>
-    <t>elc_spv_033</t>
-  </si>
-  <si>
-    <t>rez_spv_034</t>
-  </si>
-  <si>
-    <t>elc_spv_034</t>
-  </si>
-  <si>
-    <t>rez_spv_035</t>
-  </si>
-  <si>
-    <t>elc_spv_035</t>
-  </si>
-  <si>
-    <t>rez_spv_036</t>
-  </si>
-  <si>
-    <t>elc_spv_036</t>
-  </si>
-  <si>
-    <t>rez_spv_037</t>
-  </si>
-  <si>
-    <t>elc_spv_037</t>
-  </si>
-  <si>
-    <t>rez_spv_038</t>
-  </si>
-  <si>
-    <t>elc_spv_038</t>
-  </si>
-  <si>
-    <t>rez_spv_039</t>
-  </si>
-  <si>
-    <t>elc_spv_039</t>
-  </si>
-  <si>
-    <t>rez_spv_040</t>
-  </si>
-  <si>
-    <t>elc_spv_040</t>
-  </si>
-  <si>
-    <t>rez_spv_041</t>
-  </si>
-  <si>
-    <t>elc_spv_041</t>
-  </si>
-  <si>
-    <t>rez_spv_042</t>
-  </si>
-  <si>
-    <t>elc_spv_042</t>
-  </si>
-  <si>
-    <t>rez_spv_043</t>
-  </si>
-  <si>
-    <t>elc_spv_043</t>
-  </si>
-  <si>
-    <t>rez_won_001</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>rez_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>rez_won_003</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>rez_won_004</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>rez_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>rez_won_006</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>rez_won_007</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>rez_won_008</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>rez_won_009</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>rez_won_010</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>rez_won_011</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>rez_won_012</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>rez_won_013</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>rez_won_014</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>rez_won_015</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>rez_won_016</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>rez_won_017</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>rez_won_018</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>rez_won_019</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>rez_won_020</t>
-  </si>
-  <si>
-    <t>elc_won_020</t>
-  </si>
-  <si>
-    <t>rez_won_021</t>
-  </si>
-  <si>
-    <t>elc_won_021</t>
-  </si>
-  <si>
-    <t>rez_won_022</t>
-  </si>
-  <si>
-    <t>elc_won_022</t>
-  </si>
-  <si>
-    <t>rez_won_023</t>
-  </si>
-  <si>
-    <t>elc_won_023</t>
-  </si>
-  <si>
-    <t>rez_won_024</t>
-  </si>
-  <si>
-    <t>elc_won_024</t>
-  </si>
-  <si>
-    <t>rez_won_025</t>
-  </si>
-  <si>
-    <t>elc_won_025</t>
-  </si>
-  <si>
-    <t>rez_won_026</t>
-  </si>
-  <si>
-    <t>elc_won_026</t>
-  </si>
-  <si>
-    <t>rez_won_027</t>
-  </si>
-  <si>
-    <t>elc_won_027</t>
-  </si>
-  <si>
-    <t>rez_won_028</t>
-  </si>
-  <si>
-    <t>elc_won_028</t>
-  </si>
-  <si>
-    <t>rez_won_029</t>
-  </si>
-  <si>
-    <t>elc_won_029</t>
-  </si>
-  <si>
-    <t>rez_won_030</t>
-  </si>
-  <si>
-    <t>elc_won_030</t>
-  </si>
-  <si>
-    <t>rez_won_031</t>
-  </si>
-  <si>
-    <t>elc_won_031</t>
-  </si>
-  <si>
-    <t>rez_won_032</t>
-  </si>
-  <si>
-    <t>elc_won_032</t>
-  </si>
-  <si>
-    <t>rez_won_033</t>
-  </si>
-  <si>
-    <t>elc_won_033</t>
-  </si>
-  <si>
-    <t>rez_won_034</t>
-  </si>
-  <si>
-    <t>elc_won_034</t>
-  </si>
-  <si>
-    <t>rez_won_035</t>
-  </si>
-  <si>
-    <t>elc_won_035</t>
-  </si>
-  <si>
-    <t>rez_won_036</t>
-  </si>
-  <si>
-    <t>elc_won_036</t>
-  </si>
-  <si>
-    <t>rez_won_037</t>
-  </si>
-  <si>
-    <t>elc_won_037</t>
-  </si>
-  <si>
-    <t>rez_won_038</t>
-  </si>
-  <si>
-    <t>elc_won_038</t>
-  </si>
-  <si>
-    <t>rez_won_039</t>
-  </si>
-  <si>
-    <t>elc_won_039</t>
-  </si>
-  <si>
-    <t>rez_won_040</t>
-  </si>
-  <si>
-    <t>elc_won_040</t>
-  </si>
-  <si>
-    <t>rez_won_041</t>
-  </si>
-  <si>
-    <t>elc_won_041</t>
-  </si>
-  <si>
-    <t>rez_won_042</t>
-  </si>
-  <si>
-    <t>elc_won_042</t>
-  </si>
-  <si>
-    <t>rez_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>rez_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>rez_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>rez_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>rez_wof_005</t>
-  </si>
-  <si>
-    <t>elc_wof_005</t>
-  </si>
-  <si>
-    <t>rez_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>rez_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>rez_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>rez_wof_009</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>rez_wof_010</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>rez_wof_011</t>
-  </si>
-  <si>
-    <t>elc_wof_011</t>
-  </si>
-  <si>
-    <t>rez_wof_012</t>
-  </si>
-  <si>
-    <t>elc_wof_012</t>
-  </si>
-  <si>
-    <t>rez_wof_013</t>
-  </si>
-  <si>
-    <t>elc_wof_013</t>
-  </si>
-  <si>
-    <t>rez_wof_014</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>rez_wof_015</t>
-  </si>
-  <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>rez_wof_016</t>
-  </si>
-  <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>rez_wof_017</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>rez_wof_018</t>
-  </si>
-  <si>
-    <t>elc_wof_018</t>
-  </si>
-  <si>
-    <t>rez_wof_019</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
-  </si>
-  <si>
-    <t>rez_wof_020</t>
-  </si>
-  <si>
-    <t>elc_wof_020</t>
+    <t>p_w62193952-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w62193952-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w62218063-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w62218063-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w65600948-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w65600948-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w75136015-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w75136015-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w83525879-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w83525879-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w87404898-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w87404898-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w87434264-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w87434264-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w89173873-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w89173873-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w89637370-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w89637370-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w90454383-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w90454383-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w92348290-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w92348290-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w92348290-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w92348290-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w98231311-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w98231311-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w102682082-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w102682082-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w102925909-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w102925909-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w103079596-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w103079596-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w104080393-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w104080393-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w105759402-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w105759402-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w105811523-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w105811523-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w107391770-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w107391770-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w107431792-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w107431792-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w107937167-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w107937167-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w120584910-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w120584910-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w120941269-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w120941269-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w125754107-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w125754107-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w125769921-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w125769921-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w127585817-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w127585817-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w131625968-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w131625968-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w142414070-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w142414070-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w142414070-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w142414070-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w156418705-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w156418705-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w162871098-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w162871098-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w167540668-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w167540668-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w167540668-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w167540668-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w167590549-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w167590549-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w167648085-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w167648085-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w169647963-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w169647963-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w169789536-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w169789536-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w170672051-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w170672051-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w176362710-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w176362710-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w176940672-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w176940672-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w177800991-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w177800991-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w178240552-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w178240552-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w178968761-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w178968761-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w178968761-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w178968761-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w179136373-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w179136373-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w179136373-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w179136373-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w179140081-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w179140081-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w181284049-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w181284049-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w181366662-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w181366662-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w181366662-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w181366662-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w182042518-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w182042518-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w182408147-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w182408147-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w183402339-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w183402339-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w183757901-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w183757901-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w183759046-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w183759046-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w184201271-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w184201271-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w184552955-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w184552955-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w184560833-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w184560833-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w184581460-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w184581460-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w185171518-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w185171518-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w185497473-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w185497473-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w193465369-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w193465369-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w193977981-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w193977981-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w193978748-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w193978748-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w200223220-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w200223220-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w200232961-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w200232961-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w200757306-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w200757306-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w207991752-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w207991752-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w208749745-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w208749745-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w209365700-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w209365700-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w209976655-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w209976655-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w213181313-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w213181313-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w219384657-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w219384657-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w219384657-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w219384657-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w219596295-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w219596295-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w220129604-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w220129604-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w230551819-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w230551819-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w238322344-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w238322344-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w260486370-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w260486370-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w359805008-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w359805008-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w455498147-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w455498147-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w496302277-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w496302277-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w545652232-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w545652232-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w586032034-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_w586032034-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w586032034-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w586032034-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w631673098-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w631673098-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w663042845-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w663042845-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w663042849-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w663042849-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w685294883-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w685294883-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w693869805-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w693869805-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w836844162-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w836844162-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w934819484-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w934819484-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w1146812331-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w1146812331-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_w1146878078-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_w1146878078-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_r17287657-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_r17287657-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA25-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA25-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA20-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA20-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA22-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA22-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA29-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA29-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA3-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA3-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA23-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA23-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA30-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA30-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA18-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA18-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA11-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA11-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA40-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA40-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA39-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA39-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA26-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA26-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA2-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA2-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA7-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA7-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA5-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA5-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA6-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA6-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA31-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA31-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA15-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA15-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA1-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA1-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA36-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA36-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA19-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA19-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA24-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA24-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA14-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA14-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA17-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA17-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA38-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA38-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA16-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA16-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA28-765_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA28-765_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA4-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA4-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA33-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA33-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA42-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA42-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA41-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA41-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA43-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA43-400_ZAF*</t>
+  </si>
+  <si>
+    <t>p_ZA44-400_ZAF</t>
+  </si>
+  <si>
+    <t>e_ZA44-400_ZAF*</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_001</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_001</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_002</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_002</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_003</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_003</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_004</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_004</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_005</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_005</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_006</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_006</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_007</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_007</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_008</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_008</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_009</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_009</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_010</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_010</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_011</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_011</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_012</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_012</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_013</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_013</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_014</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_014</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_015</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_015</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_016</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_016</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_017</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_017</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_018</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_018</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_019</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_019</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_020</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_020</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_021</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_021</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_022</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_022</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_023</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_023</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_024</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_024</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_025</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_025</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_026</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_026</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_027</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_027</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_028</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_028</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_029</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_029</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_030</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_030</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_031</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_031</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_032</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_032</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_033</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_033</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_034</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_034</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_035</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_035</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_036</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_036</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_037</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_037</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_038</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_038</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_039</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_039</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_040</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_040</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_041</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_041</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_042</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_042</t>
+  </si>
+  <si>
+    <t>rez_spv_ZAF_043</t>
+  </si>
+  <si>
+    <t>elc_spv_ZAF_043</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_001</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_001</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_002</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_002</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_003</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_003</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_004</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_004</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_005</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_005</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_006</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_006</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_007</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_007</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_008</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_008</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_009</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_009</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_010</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_010</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_011</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_011</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_012</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_012</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_013</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_013</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_014</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_014</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_015</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_015</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_016</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_016</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_017</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_017</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_018</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_018</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_019</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_019</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_020</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_020</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_021</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_021</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_022</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_022</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_023</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_023</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_024</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_024</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_025</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_025</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_026</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_026</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_027</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_027</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_028</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_028</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_029</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_029</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_030</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_030</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_031</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_031</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_032</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_032</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_033</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_033</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_034</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_034</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_035</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_035</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_036</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_036</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_037</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_037</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_038</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_038</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_039</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_039</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_040</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_040</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_041</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_041</t>
+  </si>
+  <si>
+    <t>rez_won_ZAF_042</t>
+  </si>
+  <si>
+    <t>elc_won_ZAF_042</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_001</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_001</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_002</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_002</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_003</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_003</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_004</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_004</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_005</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_005</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_006</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_006</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_007</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_007</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_008</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_008</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_009</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_009</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_010</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_010</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_011</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_011</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_012</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_012</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_013</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_013</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_014</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_014</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_015</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_015</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_016</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_016</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_017</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_017</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_018</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_018</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_019</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_019</t>
+  </si>
+  <si>
+    <t>rez_wof_ZAF_020</t>
+  </si>
+  <si>
+    <t>elc_wof_ZAF_020</t>
   </si>
 </sst>
 </file>
@@ -2549,8 +2597,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589459FA-C2CE-4D31-BE7D-F6961E807B28}">
-  <dimension ref="B9:E237"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68FBAB-036C-4095-AAC6-30DFE22ED691}">
+  <dimension ref="B9:E245"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -5747,6 +5795,118 @@
         <v>557</v>
       </c>
       <c r="E237" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="238" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B238" t="s">
+        <v>558</v>
+      </c>
+      <c r="C238" t="s">
+        <v>559</v>
+      </c>
+      <c r="D238" t="s">
+        <v>559</v>
+      </c>
+      <c r="E238" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="239" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B239" t="s">
+        <v>560</v>
+      </c>
+      <c r="C239" t="s">
+        <v>561</v>
+      </c>
+      <c r="D239" t="s">
+        <v>561</v>
+      </c>
+      <c r="E239" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="240" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B240" t="s">
+        <v>562</v>
+      </c>
+      <c r="C240" t="s">
+        <v>563</v>
+      </c>
+      <c r="D240" t="s">
+        <v>563</v>
+      </c>
+      <c r="E240" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="241" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B241" t="s">
+        <v>564</v>
+      </c>
+      <c r="C241" t="s">
+        <v>565</v>
+      </c>
+      <c r="D241" t="s">
+        <v>565</v>
+      </c>
+      <c r="E241" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="242" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B242" t="s">
+        <v>566</v>
+      </c>
+      <c r="C242" t="s">
+        <v>567</v>
+      </c>
+      <c r="D242" t="s">
+        <v>567</v>
+      </c>
+      <c r="E242" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="243" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B243" t="s">
+        <v>568</v>
+      </c>
+      <c r="C243" t="s">
+        <v>569</v>
+      </c>
+      <c r="D243" t="s">
+        <v>569</v>
+      </c>
+      <c r="E243" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="244" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B244" t="s">
+        <v>570</v>
+      </c>
+      <c r="C244" t="s">
+        <v>571</v>
+      </c>
+      <c r="D244" t="s">
+        <v>571</v>
+      </c>
+      <c r="E244" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="245" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B245" t="s">
+        <v>572</v>
+      </c>
+      <c r="C245" t="s">
+        <v>573</v>
+      </c>
+      <c r="D245" t="s">
+        <v>573</v>
+      </c>
+      <c r="E245" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-27 08:54
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A105B0F4-A88A-43EA-80F5-2B3287B8925F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E71F3BA-034B-42CF-B182-F871D1FDA4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2597,7 +2597,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D46BE6B-4719-4430-B9EF-53C34C6F42BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC56E9B5-49E1-42CB-A240-FDD4911E0C82}">
   <dimension ref="B9:E245"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Unit comm parameters for coal ccs
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/Sets-vervestacks.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E71F3BA-034B-42CF-B182-F871D1FDA4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
-    <sheet name="geo_sets" sheetId="3" r:id="rId2"/>
-    <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId3"/>
+    <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId3"/>
+    <sheet name="geo_sets" sheetId="3" r:id="rId4"/>
+    <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId5"/>
+    <sheet name="SetsEditor- Proc" sheetId="4" r:id="rId6"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="586">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -1760,19 +1761,61 @@
   </si>
   <si>
     <t>elc_wof_ZAF_020</t>
+  </si>
+  <si>
+    <t>~TFM_PSets</t>
+  </si>
+  <si>
+    <t>t_pos_andor_forsets</t>
+  </si>
+  <si>
+    <t>t_neg_andor_forsets</t>
+  </si>
+  <si>
+    <t>t_neg_andor</t>
+  </si>
+  <si>
+    <t>setdesc</t>
+  </si>
+  <si>
+    <t>pset_set</t>
+  </si>
+  <si>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>pset_pd</t>
+  </si>
+  <si>
+    <t>coal_ccs</t>
+  </si>
+  <si>
+    <t>Coal CCS</t>
+  </si>
+  <si>
+    <t>-ep*</t>
+  </si>
+  <si>
+    <t>coal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1812,38 +1855,130 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.49995422223578601"/>
+        <color theme="4" tint="0.499949991703033"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
+        <color theme="4" tint="0.399980008602142"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="20"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="21"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="2" builtinId="18"/>
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Heading 2" xfId="20" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="21" builtinId="18"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2151,27 +2286,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.57142857142857" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.57142857142857" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.85714285714286" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42857142857143" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.71428571428571" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" ht="14.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="14.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2197,22 +2332,22 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:11" ht="14.25">
       <c r="B3" t="str">
         <f>"e_*"&amp;K3</f>
         <v>e_*220</v>
       </c>
       <c r="D3" t="str">
-        <f t="shared" ref="D3:D23" si="0">"Elec-"&amp;K3&amp;"V"</f>
+        <f t="shared" si="0" ref="D3:D23">"Elec-"&amp;K3&amp;"V"</f>
         <v>Elec-220V</v>
       </c>
       <c r="K3">
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:11" ht="14.25">
       <c r="B4" t="str">
-        <f t="shared" ref="B4:B23" si="1">"e_*"&amp;K4</f>
+        <f t="shared" si="1" ref="B4:B23">"e_*"&amp;K4</f>
         <v>e_*400</v>
       </c>
       <c r="D4" t="str">
@@ -2223,7 +2358,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:11" ht="14.25">
       <c r="B5" t="str">
         <f t="shared" si="1"/>
         <v>e_*380</v>
@@ -2236,7 +2371,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:11" ht="14.25">
       <c r="B6" t="str">
         <f t="shared" si="1"/>
         <v>e_*225</v>
@@ -2249,7 +2384,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:11" ht="14.25">
       <c r="B7" t="str">
         <f t="shared" si="1"/>
         <v>e_*330</v>
@@ -2262,7 +2397,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:11" ht="14.25">
       <c r="B8" t="str">
         <f t="shared" si="1"/>
         <v>e_*275</v>
@@ -2275,7 +2410,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:11" ht="14.25">
       <c r="B9" t="str">
         <f t="shared" si="1"/>
         <v>e_*420</v>
@@ -2288,7 +2423,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:11" ht="14.25">
       <c r="B10" t="str">
         <f t="shared" si="1"/>
         <v>e_*300</v>
@@ -2301,7 +2436,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:11" ht="14.25">
       <c r="B11" t="str">
         <f t="shared" si="1"/>
         <v>e_*500</v>
@@ -2314,7 +2449,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:11" ht="14.25">
       <c r="B12" t="str">
         <f t="shared" si="1"/>
         <v>e_*750</v>
@@ -2327,7 +2462,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:11" ht="14.25">
       <c r="B13" t="str">
         <f t="shared" si="1"/>
         <v>e_*450</v>
@@ -2340,7 +2475,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:11" ht="14.25">
       <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v>e_*515</v>
@@ -2353,7 +2488,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:11" ht="14.25">
       <c r="B15" t="str">
         <f t="shared" si="1"/>
         <v>e_*525</v>
@@ -2366,7 +2501,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:11" ht="14.25">
       <c r="B16" t="str">
         <f t="shared" si="1"/>
         <v>e_*320</v>
@@ -2379,7 +2514,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:11" ht="14.25">
       <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v>e_*150</v>
@@ -2392,7 +2527,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:11" ht="14.25">
       <c r="B18" t="str">
         <f t="shared" si="1"/>
         <v>e_*270</v>
@@ -2405,7 +2540,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:11" ht="14.25">
       <c r="B19" t="str">
         <f t="shared" si="1"/>
         <v>e_*350</v>
@@ -2418,7 +2553,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:11" ht="14.25">
       <c r="B20" t="str">
         <f t="shared" si="1"/>
         <v>e_*250</v>
@@ -2431,7 +2566,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:11" ht="14.25">
       <c r="B21" t="str">
         <f t="shared" si="1"/>
         <v>e_*200</v>
@@ -2444,7 +2579,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:11" ht="14.25">
       <c r="B22" t="str">
         <f t="shared" si="1"/>
         <v>e_*236</v>
@@ -2457,7 +2592,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:11" ht="14.25">
       <c r="B23" t="str">
         <f t="shared" si="1"/>
         <v>e_*600</v>
@@ -2470,7 +2605,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:4" ht="14.25">
       <c r="B24" t="s">
         <v>44</v>
       </c>
@@ -2478,7 +2613,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:4" ht="14.25">
       <c r="B25" t="s">
         <v>45</v>
       </c>
@@ -2486,7 +2621,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:4" ht="14.25">
       <c r="B26" t="s">
         <v>60</v>
       </c>
@@ -2494,7 +2629,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:4" ht="14.25">
       <c r="B27" t="s">
         <v>61</v>
       </c>
@@ -2502,7 +2637,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:4" ht="14.25">
       <c r="B28" t="s">
         <v>46</v>
       </c>
@@ -2511,7 +2646,7 @@
         <v>bioenergy</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:4" ht="14.25">
       <c r="B29" t="s">
         <v>47</v>
       </c>
@@ -2520,7 +2655,7 @@
         <v>hydrogen</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:4" ht="14.25">
       <c r="B30" t="s">
         <v>36</v>
       </c>
@@ -2529,7 +2664,7 @@
         <v>nuclear</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:4" ht="14.25">
       <c r="B31" t="s">
         <v>48</v>
       </c>
@@ -2538,7 +2673,7 @@
         <v>ELC</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:4" ht="14.25">
       <c r="B32" t="s">
         <v>49</v>
       </c>
@@ -2546,7 +2681,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:4" ht="14.25">
       <c r="B33" t="s">
         <v>50</v>
       </c>
@@ -2554,7 +2689,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:4" ht="14.25">
       <c r="B34" t="s">
         <v>51</v>
       </c>
@@ -2562,7 +2697,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:4" ht="14.25">
       <c r="B35" t="s">
         <v>52</v>
       </c>
@@ -2570,7 +2705,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:4" ht="14.25">
       <c r="B36" t="s">
         <v>53</v>
       </c>
@@ -2579,7 +2714,7 @@
         <v>co2</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:4" ht="14.25">
       <c r="B37" t="s">
         <v>54</v>
       </c>
@@ -2589,24 +2724,24 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A26:D37">
-    <sortCondition ref="A26:A37"/>
+  <sortState ref="A26:D37">
+    <sortCondition sortBy="value" ref="A26:A37"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC56E9B5-49E1-42CB-A240-FDD4911E0C82}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8F5E3B7-6D2D-417D-9024-AF746429CD6E}">
   <dimension ref="B9:E245"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:2" ht="14.25">
       <c r="B9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:5" ht="14.25">
       <c r="B10" t="s">
         <v>99</v>
       </c>
@@ -2620,7 +2755,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:5" ht="14.25">
       <c r="B11" t="s">
         <v>103</v>
       </c>
@@ -2634,7 +2769,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:5" ht="14.25">
       <c r="B12" t="s">
         <v>106</v>
       </c>
@@ -2648,7 +2783,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:5" ht="14.25">
       <c r="B13" t="s">
         <v>108</v>
       </c>
@@ -2662,7 +2797,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:5" ht="14.25">
       <c r="B14" t="s">
         <v>110</v>
       </c>
@@ -2676,7 +2811,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:5" ht="14.25">
       <c r="B15" t="s">
         <v>112</v>
       </c>
@@ -2690,7 +2825,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:5" ht="14.25">
       <c r="B16" t="s">
         <v>114</v>
       </c>
@@ -2704,7 +2839,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:5" ht="14.25">
       <c r="B17" t="s">
         <v>116</v>
       </c>
@@ -2718,7 +2853,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:5" ht="14.25">
       <c r="B18" t="s">
         <v>118</v>
       </c>
@@ -2732,7 +2867,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:5" ht="14.25">
       <c r="B19" t="s">
         <v>120</v>
       </c>
@@ -2746,7 +2881,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:5" ht="14.25">
       <c r="B20" t="s">
         <v>122</v>
       </c>
@@ -2760,7 +2895,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:5" ht="14.25">
       <c r="B21" t="s">
         <v>124</v>
       </c>
@@ -2774,7 +2909,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:5" ht="14.25">
       <c r="B22" t="s">
         <v>126</v>
       </c>
@@ -2788,7 +2923,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:5" ht="14.25">
       <c r="B23" t="s">
         <v>128</v>
       </c>
@@ -2802,7 +2937,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:5" ht="14.25">
       <c r="B24" t="s">
         <v>130</v>
       </c>
@@ -2816,7 +2951,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:5" ht="14.25">
       <c r="B25" t="s">
         <v>132</v>
       </c>
@@ -2830,7 +2965,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:5" ht="14.25">
       <c r="B26" t="s">
         <v>134</v>
       </c>
@@ -2844,7 +2979,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:5" ht="14.25">
       <c r="B27" t="s">
         <v>136</v>
       </c>
@@ -2858,7 +2993,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:5" ht="14.25">
       <c r="B28" t="s">
         <v>138</v>
       </c>
@@ -2872,7 +3007,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:5" ht="14.25">
       <c r="B29" t="s">
         <v>140</v>
       </c>
@@ -2886,7 +3021,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:5" ht="14.25">
       <c r="B30" t="s">
         <v>142</v>
       </c>
@@ -2900,7 +3035,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:5" ht="14.25">
       <c r="B31" t="s">
         <v>144</v>
       </c>
@@ -2914,7 +3049,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:5" ht="14.25">
       <c r="B32" t="s">
         <v>146</v>
       </c>
@@ -2928,7 +3063,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:5" ht="14.25">
       <c r="B33" t="s">
         <v>148</v>
       </c>
@@ -2942,7 +3077,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:5" ht="14.25">
       <c r="B34" t="s">
         <v>150</v>
       </c>
@@ -2956,7 +3091,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:5" ht="14.25">
       <c r="B35" t="s">
         <v>152</v>
       </c>
@@ -2970,7 +3105,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:5" ht="14.25">
       <c r="B36" t="s">
         <v>154</v>
       </c>
@@ -2984,7 +3119,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:5" ht="14.25">
       <c r="B37" t="s">
         <v>156</v>
       </c>
@@ -2998,7 +3133,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:5" ht="14.25">
       <c r="B38" t="s">
         <v>158</v>
       </c>
@@ -3012,7 +3147,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:5" ht="14.25">
       <c r="B39" t="s">
         <v>160</v>
       </c>
@@ -3026,7 +3161,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:5" ht="14.25">
       <c r="B40" t="s">
         <v>162</v>
       </c>
@@ -3040,7 +3175,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:5" ht="14.25">
       <c r="B41" t="s">
         <v>164</v>
       </c>
@@ -3054,7 +3189,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:5" ht="14.25">
       <c r="B42" t="s">
         <v>166</v>
       </c>
@@ -3068,7 +3203,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:5" ht="14.25">
       <c r="B43" t="s">
         <v>168</v>
       </c>
@@ -3082,7 +3217,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:5" ht="14.25">
       <c r="B44" t="s">
         <v>170</v>
       </c>
@@ -3096,7 +3231,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:5" ht="14.25">
       <c r="B45" t="s">
         <v>172</v>
       </c>
@@ -3110,7 +3245,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:5" ht="14.25">
       <c r="B46" t="s">
         <v>174</v>
       </c>
@@ -3124,7 +3259,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:5" ht="14.25">
       <c r="B47" t="s">
         <v>176</v>
       </c>
@@ -3138,7 +3273,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:5" ht="14.25">
       <c r="B48" t="s">
         <v>178</v>
       </c>
@@ -3152,7 +3287,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:5" ht="14.25">
       <c r="B49" t="s">
         <v>180</v>
       </c>
@@ -3166,7 +3301,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:5" ht="14.25">
       <c r="B50" t="s">
         <v>182</v>
       </c>
@@ -3180,7 +3315,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="51" spans="2:5" ht="14.25">
       <c r="B51" t="s">
         <v>184</v>
       </c>
@@ -3194,7 +3329,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:5" ht="14.25">
       <c r="B52" t="s">
         <v>186</v>
       </c>
@@ -3208,7 +3343,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:5" ht="14.25">
       <c r="B53" t="s">
         <v>188</v>
       </c>
@@ -3222,7 +3357,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:5" ht="14.25">
       <c r="B54" t="s">
         <v>190</v>
       </c>
@@ -3236,7 +3371,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:5" ht="14.25">
       <c r="B55" t="s">
         <v>192</v>
       </c>
@@ -3250,7 +3385,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:5" ht="14.25">
       <c r="B56" t="s">
         <v>194</v>
       </c>
@@ -3264,7 +3399,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:5" ht="14.25">
       <c r="B57" t="s">
         <v>196</v>
       </c>
@@ -3278,7 +3413,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:5" ht="14.25">
       <c r="B58" t="s">
         <v>198</v>
       </c>
@@ -3292,7 +3427,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:5" ht="14.25">
       <c r="B59" t="s">
         <v>200</v>
       </c>
@@ -3306,7 +3441,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:5" ht="14.25">
       <c r="B60" t="s">
         <v>202</v>
       </c>
@@ -3320,7 +3455,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:5" ht="14.25">
       <c r="B61" t="s">
         <v>204</v>
       </c>
@@ -3334,7 +3469,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:5" ht="14.25">
       <c r="B62" t="s">
         <v>206</v>
       </c>
@@ -3348,7 +3483,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:5" ht="14.25">
       <c r="B63" t="s">
         <v>208</v>
       </c>
@@ -3362,7 +3497,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:5" ht="14.25">
       <c r="B64" t="s">
         <v>210</v>
       </c>
@@ -3376,7 +3511,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:5" ht="14.25">
       <c r="B65" t="s">
         <v>212</v>
       </c>
@@ -3390,7 +3525,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:5" ht="14.25">
       <c r="B66" t="s">
         <v>214</v>
       </c>
@@ -3404,7 +3539,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:5" ht="14.25">
       <c r="B67" t="s">
         <v>216</v>
       </c>
@@ -3418,7 +3553,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:5" ht="14.25">
       <c r="B68" t="s">
         <v>218</v>
       </c>
@@ -3432,7 +3567,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:5" ht="14.25">
       <c r="B69" t="s">
         <v>220</v>
       </c>
@@ -3446,7 +3581,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:5" ht="14.25">
       <c r="B70" t="s">
         <v>222</v>
       </c>
@@ -3460,7 +3595,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:5" ht="14.25">
       <c r="B71" t="s">
         <v>224</v>
       </c>
@@ -3474,7 +3609,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:5" ht="14.25">
       <c r="B72" t="s">
         <v>226</v>
       </c>
@@ -3488,7 +3623,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:5" ht="14.25">
       <c r="B73" t="s">
         <v>228</v>
       </c>
@@ -3502,7 +3637,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:5" ht="14.25">
       <c r="B74" t="s">
         <v>230</v>
       </c>
@@ -3516,7 +3651,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="75" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:5" ht="14.25">
       <c r="B75" t="s">
         <v>232</v>
       </c>
@@ -3530,7 +3665,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:5" ht="14.25">
       <c r="B76" t="s">
         <v>234</v>
       </c>
@@ -3544,7 +3679,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:5" ht="14.25">
       <c r="B77" t="s">
         <v>236</v>
       </c>
@@ -3558,7 +3693,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:5" ht="14.25">
       <c r="B78" t="s">
         <v>238</v>
       </c>
@@ -3572,7 +3707,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:5" ht="14.25">
       <c r="B79" t="s">
         <v>240</v>
       </c>
@@ -3586,7 +3721,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:5" ht="14.25">
       <c r="B80" t="s">
         <v>242</v>
       </c>
@@ -3600,7 +3735,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:5" ht="14.25">
       <c r="B81" t="s">
         <v>244</v>
       </c>
@@ -3614,7 +3749,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="82" spans="2:5" ht="14.25">
       <c r="B82" t="s">
         <v>246</v>
       </c>
@@ -3628,7 +3763,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:5" ht="14.25">
       <c r="B83" t="s">
         <v>248</v>
       </c>
@@ -3642,7 +3777,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="84" spans="2:5" ht="14.25">
       <c r="B84" t="s">
         <v>250</v>
       </c>
@@ -3656,7 +3791,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="85" spans="2:5" ht="14.25">
       <c r="B85" t="s">
         <v>252</v>
       </c>
@@ -3670,7 +3805,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="86" spans="2:5" ht="14.25">
       <c r="B86" t="s">
         <v>254</v>
       </c>
@@ -3684,7 +3819,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="87" spans="2:5" ht="14.25">
       <c r="B87" t="s">
         <v>256</v>
       </c>
@@ -3698,7 +3833,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="88" spans="2:5" ht="14.25">
       <c r="B88" t="s">
         <v>258</v>
       </c>
@@ -3712,7 +3847,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="89" spans="2:5" ht="14.25">
       <c r="B89" t="s">
         <v>260</v>
       </c>
@@ -3726,7 +3861,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="90" spans="2:5" ht="14.25">
       <c r="B90" t="s">
         <v>262</v>
       </c>
@@ -3740,7 +3875,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="91" spans="2:5" ht="14.25">
       <c r="B91" t="s">
         <v>264</v>
       </c>
@@ -3754,7 +3889,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="92" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="92" spans="2:5" ht="14.25">
       <c r="B92" t="s">
         <v>266</v>
       </c>
@@ -3768,7 +3903,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="93" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="93" spans="2:5" ht="14.25">
       <c r="B93" t="s">
         <v>268</v>
       </c>
@@ -3782,7 +3917,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="94" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="94" spans="2:5" ht="14.25">
       <c r="B94" t="s">
         <v>270</v>
       </c>
@@ -3796,7 +3931,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="95" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="95" spans="2:5" ht="14.25">
       <c r="B95" t="s">
         <v>272</v>
       </c>
@@ -3810,7 +3945,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="96" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="96" spans="2:5" ht="14.25">
       <c r="B96" t="s">
         <v>274</v>
       </c>
@@ -3824,7 +3959,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="97" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="97" spans="2:5" ht="14.25">
       <c r="B97" t="s">
         <v>276</v>
       </c>
@@ -3838,7 +3973,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="98" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="98" spans="2:5" ht="14.25">
       <c r="B98" t="s">
         <v>278</v>
       </c>
@@ -3852,7 +3987,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="99" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="99" spans="2:5" ht="14.25">
       <c r="B99" t="s">
         <v>280</v>
       </c>
@@ -3866,7 +4001,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="100" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="100" spans="2:5" ht="14.25">
       <c r="B100" t="s">
         <v>282</v>
       </c>
@@ -3880,7 +4015,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="101" spans="2:5" ht="14.25">
       <c r="B101" t="s">
         <v>284</v>
       </c>
@@ -3894,7 +4029,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="102" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="102" spans="2:5" ht="14.25">
       <c r="B102" t="s">
         <v>286</v>
       </c>
@@ -3908,7 +4043,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="103" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="103" spans="2:5" ht="14.25">
       <c r="B103" t="s">
         <v>288</v>
       </c>
@@ -3922,7 +4057,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="104" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="104" spans="2:5" ht="14.25">
       <c r="B104" t="s">
         <v>290</v>
       </c>
@@ -3936,7 +4071,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="105" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="105" spans="2:5" ht="14.25">
       <c r="B105" t="s">
         <v>292</v>
       </c>
@@ -3950,7 +4085,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="106" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="106" spans="2:5" ht="14.25">
       <c r="B106" t="s">
         <v>294</v>
       </c>
@@ -3964,7 +4099,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="107" spans="2:5" ht="14.25">
       <c r="B107" t="s">
         <v>296</v>
       </c>
@@ -3978,7 +4113,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="108" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="108" spans="2:5" ht="14.25">
       <c r="B108" t="s">
         <v>298</v>
       </c>
@@ -3992,7 +4127,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="109" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="109" spans="2:5" ht="14.25">
       <c r="B109" t="s">
         <v>300</v>
       </c>
@@ -4006,7 +4141,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="110" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="110" spans="2:5" ht="14.25">
       <c r="B110" t="s">
         <v>302</v>
       </c>
@@ -4020,7 +4155,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="111" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="111" spans="2:5" ht="14.25">
       <c r="B111" t="s">
         <v>304</v>
       </c>
@@ -4034,7 +4169,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="112" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="112" spans="2:5" ht="14.25">
       <c r="B112" t="s">
         <v>306</v>
       </c>
@@ -4048,7 +4183,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="113" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="113" spans="2:5" ht="14.25">
       <c r="B113" t="s">
         <v>308</v>
       </c>
@@ -4062,7 +4197,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="114" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="114" spans="2:5" ht="14.25">
       <c r="B114" t="s">
         <v>310</v>
       </c>
@@ -4076,7 +4211,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="115" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="115" spans="2:5" ht="14.25">
       <c r="B115" t="s">
         <v>312</v>
       </c>
@@ -4090,7 +4225,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="116" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="116" spans="2:5" ht="14.25">
       <c r="B116" t="s">
         <v>314</v>
       </c>
@@ -4104,7 +4239,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="117" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="117" spans="2:5" ht="14.25">
       <c r="B117" t="s">
         <v>316</v>
       </c>
@@ -4118,7 +4253,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="118" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="118" spans="2:5" ht="14.25">
       <c r="B118" t="s">
         <v>318</v>
       </c>
@@ -4132,7 +4267,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="119" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="119" spans="2:5" ht="14.25">
       <c r="B119" t="s">
         <v>320</v>
       </c>
@@ -4146,7 +4281,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="120" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="120" spans="2:5" ht="14.25">
       <c r="B120" t="s">
         <v>322</v>
       </c>
@@ -4160,7 +4295,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="121" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="121" spans="2:5" ht="14.25">
       <c r="B121" t="s">
         <v>324</v>
       </c>
@@ -4174,7 +4309,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="122" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="122" spans="2:5" ht="14.25">
       <c r="B122" t="s">
         <v>326</v>
       </c>
@@ -4188,7 +4323,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="123" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="123" spans="2:5" ht="14.25">
       <c r="B123" t="s">
         <v>328</v>
       </c>
@@ -4202,7 +4337,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="124" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="124" spans="2:5" ht="14.25">
       <c r="B124" t="s">
         <v>330</v>
       </c>
@@ -4216,7 +4351,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="125" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="125" spans="2:5" ht="14.25">
       <c r="B125" t="s">
         <v>332</v>
       </c>
@@ -4230,7 +4365,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="126" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="126" spans="2:5" ht="14.25">
       <c r="B126" t="s">
         <v>334</v>
       </c>
@@ -4244,7 +4379,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="127" spans="2:5" ht="14.25">
       <c r="B127" t="s">
         <v>336</v>
       </c>
@@ -4258,7 +4393,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="128" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="128" spans="2:5" ht="14.25">
       <c r="B128" t="s">
         <v>338</v>
       </c>
@@ -4272,7 +4407,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="129" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="129" spans="2:5" ht="14.25">
       <c r="B129" t="s">
         <v>340</v>
       </c>
@@ -4286,7 +4421,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="130" spans="2:5" ht="14.25">
       <c r="B130" t="s">
         <v>342</v>
       </c>
@@ -4300,7 +4435,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="131" spans="2:5" ht="14.25">
       <c r="B131" t="s">
         <v>344</v>
       </c>
@@ -4314,7 +4449,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="132" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="132" spans="2:5" ht="14.25">
       <c r="B132" t="s">
         <v>346</v>
       </c>
@@ -4328,7 +4463,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="133" spans="2:5" ht="14.25">
       <c r="B133" t="s">
         <v>348</v>
       </c>
@@ -4342,7 +4477,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="134" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="134" spans="2:5" ht="14.25">
       <c r="B134" t="s">
         <v>350</v>
       </c>
@@ -4356,7 +4491,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="135" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="135" spans="2:5" ht="14.25">
       <c r="B135" t="s">
         <v>352</v>
       </c>
@@ -4370,7 +4505,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="136" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="136" spans="2:5" ht="14.25">
       <c r="B136" t="s">
         <v>354</v>
       </c>
@@ -4384,7 +4519,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="137" spans="2:5" ht="14.25">
       <c r="B137" t="s">
         <v>356</v>
       </c>
@@ -4398,7 +4533,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="138" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="138" spans="2:5" ht="14.25">
       <c r="B138" t="s">
         <v>358</v>
       </c>
@@ -4412,7 +4547,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="139" spans="2:5" ht="14.25">
       <c r="B139" t="s">
         <v>360</v>
       </c>
@@ -4426,7 +4561,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="140" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="140" spans="2:5" ht="14.25">
       <c r="B140" t="s">
         <v>362</v>
       </c>
@@ -4440,7 +4575,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="141" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="141" spans="2:5" ht="14.25">
       <c r="B141" t="s">
         <v>364</v>
       </c>
@@ -4454,7 +4589,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="142" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="142" spans="2:5" ht="14.25">
       <c r="B142" t="s">
         <v>366</v>
       </c>
@@ -4468,7 +4603,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="143" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="143" spans="2:5" ht="14.25">
       <c r="B143" t="s">
         <v>368</v>
       </c>
@@ -4482,7 +4617,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="144" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="144" spans="2:5" ht="14.25">
       <c r="B144" t="s">
         <v>370</v>
       </c>
@@ -4496,7 +4631,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="145" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="145" spans="2:5" ht="14.25">
       <c r="B145" t="s">
         <v>372</v>
       </c>
@@ -4510,7 +4645,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="146" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="146" spans="2:5" ht="14.25">
       <c r="B146" t="s">
         <v>374</v>
       </c>
@@ -4524,7 +4659,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="147" spans="2:5" ht="14.25">
       <c r="B147" t="s">
         <v>376</v>
       </c>
@@ -4538,7 +4673,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="148" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="148" spans="2:5" ht="14.25">
       <c r="B148" t="s">
         <v>378</v>
       </c>
@@ -4552,7 +4687,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="149" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="149" spans="2:5" ht="14.25">
       <c r="B149" t="s">
         <v>380</v>
       </c>
@@ -4566,7 +4701,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="150" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="150" spans="2:5" ht="14.25">
       <c r="B150" t="s">
         <v>382</v>
       </c>
@@ -4580,7 +4715,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="151" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="151" spans="2:5" ht="14.25">
       <c r="B151" t="s">
         <v>384</v>
       </c>
@@ -4594,7 +4729,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="152" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="152" spans="2:5" ht="14.25">
       <c r="B152" t="s">
         <v>386</v>
       </c>
@@ -4608,7 +4743,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="153" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="153" spans="2:5" ht="14.25">
       <c r="B153" t="s">
         <v>388</v>
       </c>
@@ -4622,7 +4757,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="154" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="154" spans="2:5" ht="14.25">
       <c r="B154" t="s">
         <v>390</v>
       </c>
@@ -4636,7 +4771,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="155" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="155" spans="2:5" ht="14.25">
       <c r="B155" t="s">
         <v>392</v>
       </c>
@@ -4650,7 +4785,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="156" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="156" spans="2:5" ht="14.25">
       <c r="B156" t="s">
         <v>394</v>
       </c>
@@ -4664,7 +4799,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="157" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="157" spans="2:5" ht="14.25">
       <c r="B157" t="s">
         <v>396</v>
       </c>
@@ -4678,7 +4813,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="158" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="158" spans="2:5" ht="14.25">
       <c r="B158" t="s">
         <v>398</v>
       </c>
@@ -4692,7 +4827,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="159" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="159" spans="2:5" ht="14.25">
       <c r="B159" t="s">
         <v>400</v>
       </c>
@@ -4706,7 +4841,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="160" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="160" spans="2:5" ht="14.25">
       <c r="B160" t="s">
         <v>402</v>
       </c>
@@ -4720,7 +4855,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="161" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="161" spans="2:5" ht="14.25">
       <c r="B161" t="s">
         <v>404</v>
       </c>
@@ -4734,7 +4869,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="162" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="162" spans="2:5" ht="14.25">
       <c r="B162" t="s">
         <v>406</v>
       </c>
@@ -4748,7 +4883,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="163" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="163" spans="2:5" ht="14.25">
       <c r="B163" t="s">
         <v>408</v>
       </c>
@@ -4762,7 +4897,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="164" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="164" spans="2:5" ht="14.25">
       <c r="B164" t="s">
         <v>410</v>
       </c>
@@ -4776,7 +4911,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="165" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="165" spans="2:5" ht="14.25">
       <c r="B165" t="s">
         <v>412</v>
       </c>
@@ -4790,7 +4925,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="166" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="166" spans="2:5" ht="14.25">
       <c r="B166" t="s">
         <v>414</v>
       </c>
@@ -4804,7 +4939,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="167" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="167" spans="2:5" ht="14.25">
       <c r="B167" t="s">
         <v>416</v>
       </c>
@@ -4818,7 +4953,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="168" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="168" spans="2:5" ht="14.25">
       <c r="B168" t="s">
         <v>418</v>
       </c>
@@ -4832,7 +4967,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="169" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="169" spans="2:5" ht="14.25">
       <c r="B169" t="s">
         <v>420</v>
       </c>
@@ -4846,7 +4981,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="170" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="170" spans="2:5" ht="14.25">
       <c r="B170" t="s">
         <v>422</v>
       </c>
@@ -4860,7 +4995,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="171" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="171" spans="2:5" ht="14.25">
       <c r="B171" t="s">
         <v>424</v>
       </c>
@@ -4874,7 +5009,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="172" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="172" spans="2:5" ht="14.25">
       <c r="B172" t="s">
         <v>426</v>
       </c>
@@ -4888,7 +5023,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="173" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="173" spans="2:5" ht="14.25">
       <c r="B173" t="s">
         <v>428</v>
       </c>
@@ -4902,7 +5037,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="174" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="174" spans="2:5" ht="14.25">
       <c r="B174" t="s">
         <v>430</v>
       </c>
@@ -4916,7 +5051,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="175" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="175" spans="2:5" ht="14.25">
       <c r="B175" t="s">
         <v>432</v>
       </c>
@@ -4930,7 +5065,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="176" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="176" spans="2:5" ht="14.25">
       <c r="B176" t="s">
         <v>434</v>
       </c>
@@ -4944,7 +5079,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="177" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="177" spans="2:5" ht="14.25">
       <c r="B177" t="s">
         <v>436</v>
       </c>
@@ -4958,7 +5093,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="178" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="178" spans="2:5" ht="14.25">
       <c r="B178" t="s">
         <v>438</v>
       </c>
@@ -4972,7 +5107,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="179" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="179" spans="2:5" ht="14.25">
       <c r="B179" t="s">
         <v>440</v>
       </c>
@@ -4986,7 +5121,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="180" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="180" spans="2:5" ht="14.25">
       <c r="B180" t="s">
         <v>442</v>
       </c>
@@ -5000,7 +5135,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="181" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="181" spans="2:5" ht="14.25">
       <c r="B181" t="s">
         <v>444</v>
       </c>
@@ -5014,7 +5149,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="182" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="182" spans="2:5" ht="14.25">
       <c r="B182" t="s">
         <v>446</v>
       </c>
@@ -5028,7 +5163,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="183" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="183" spans="2:5" ht="14.25">
       <c r="B183" t="s">
         <v>448</v>
       </c>
@@ -5042,7 +5177,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="184" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="184" spans="2:5" ht="14.25">
       <c r="B184" t="s">
         <v>450</v>
       </c>
@@ -5056,7 +5191,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="185" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="185" spans="2:5" ht="14.25">
       <c r="B185" t="s">
         <v>452</v>
       </c>
@@ -5070,7 +5205,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="186" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="186" spans="2:5" ht="14.25">
       <c r="B186" t="s">
         <v>454</v>
       </c>
@@ -5084,7 +5219,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="187" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="187" spans="2:5" ht="14.25">
       <c r="B187" t="s">
         <v>456</v>
       </c>
@@ -5098,7 +5233,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="188" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="188" spans="2:5" ht="14.25">
       <c r="B188" t="s">
         <v>458</v>
       </c>
@@ -5112,7 +5247,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="189" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="189" spans="2:5" ht="14.25">
       <c r="B189" t="s">
         <v>460</v>
       </c>
@@ -5126,7 +5261,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="190" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="190" spans="2:5" ht="14.25">
       <c r="B190" t="s">
         <v>462</v>
       </c>
@@ -5140,7 +5275,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="191" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="191" spans="2:5" ht="14.25">
       <c r="B191" t="s">
         <v>464</v>
       </c>
@@ -5154,7 +5289,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="192" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="192" spans="2:5" ht="14.25">
       <c r="B192" t="s">
         <v>466</v>
       </c>
@@ -5168,7 +5303,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="193" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="193" spans="2:5" ht="14.25">
       <c r="B193" t="s">
         <v>468</v>
       </c>
@@ -5182,7 +5317,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="194" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="194" spans="2:5" ht="14.25">
       <c r="B194" t="s">
         <v>470</v>
       </c>
@@ -5196,7 +5331,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="195" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="195" spans="2:5" ht="14.25">
       <c r="B195" t="s">
         <v>472</v>
       </c>
@@ -5210,7 +5345,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="196" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="196" spans="2:5" ht="14.25">
       <c r="B196" t="s">
         <v>474</v>
       </c>
@@ -5224,7 +5359,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="197" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="197" spans="2:5" ht="14.25">
       <c r="B197" t="s">
         <v>476</v>
       </c>
@@ -5238,7 +5373,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="198" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="198" spans="2:5" ht="14.25">
       <c r="B198" t="s">
         <v>478</v>
       </c>
@@ -5252,7 +5387,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="199" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="199" spans="2:5" ht="14.25">
       <c r="B199" t="s">
         <v>480</v>
       </c>
@@ -5266,7 +5401,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="200" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="200" spans="2:5" ht="14.25">
       <c r="B200" t="s">
         <v>482</v>
       </c>
@@ -5280,7 +5415,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="201" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="201" spans="2:5" ht="14.25">
       <c r="B201" t="s">
         <v>484</v>
       </c>
@@ -5294,7 +5429,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="202" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="202" spans="2:5" ht="14.25">
       <c r="B202" t="s">
         <v>486</v>
       </c>
@@ -5308,7 +5443,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="203" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="203" spans="2:5" ht="14.25">
       <c r="B203" t="s">
         <v>488</v>
       </c>
@@ -5322,7 +5457,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="204" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="204" spans="2:5" ht="14.25">
       <c r="B204" t="s">
         <v>490</v>
       </c>
@@ -5336,7 +5471,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="205" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="205" spans="2:5" ht="14.25">
       <c r="B205" t="s">
         <v>492</v>
       </c>
@@ -5350,7 +5485,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="206" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="206" spans="2:5" ht="14.25">
       <c r="B206" t="s">
         <v>494</v>
       </c>
@@ -5364,7 +5499,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="207" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="207" spans="2:5" ht="14.25">
       <c r="B207" t="s">
         <v>496</v>
       </c>
@@ -5378,7 +5513,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="208" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="208" spans="2:5" ht="14.25">
       <c r="B208" t="s">
         <v>498</v>
       </c>
@@ -5392,7 +5527,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="209" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="209" spans="2:5" ht="14.25">
       <c r="B209" t="s">
         <v>500</v>
       </c>
@@ -5406,7 +5541,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="210" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="210" spans="2:5" ht="14.25">
       <c r="B210" t="s">
         <v>502</v>
       </c>
@@ -5420,7 +5555,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="211" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="211" spans="2:5" ht="14.25">
       <c r="B211" t="s">
         <v>504</v>
       </c>
@@ -5434,7 +5569,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="212" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="212" spans="2:5" ht="14.25">
       <c r="B212" t="s">
         <v>506</v>
       </c>
@@ -5448,7 +5583,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="213" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="213" spans="2:5" ht="14.25">
       <c r="B213" t="s">
         <v>508</v>
       </c>
@@ -5462,7 +5597,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="214" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="214" spans="2:5" ht="14.25">
       <c r="B214" t="s">
         <v>510</v>
       </c>
@@ -5476,7 +5611,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="215" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="215" spans="2:5" ht="14.25">
       <c r="B215" t="s">
         <v>512</v>
       </c>
@@ -5490,7 +5625,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="216" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="216" spans="2:5" ht="14.25">
       <c r="B216" t="s">
         <v>514</v>
       </c>
@@ -5504,7 +5639,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="217" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="217" spans="2:5" ht="14.25">
       <c r="B217" t="s">
         <v>516</v>
       </c>
@@ -5518,7 +5653,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="218" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="218" spans="2:5" ht="14.25">
       <c r="B218" t="s">
         <v>518</v>
       </c>
@@ -5532,7 +5667,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="219" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="219" spans="2:5" ht="14.25">
       <c r="B219" t="s">
         <v>520</v>
       </c>
@@ -5546,7 +5681,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="220" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="220" spans="2:5" ht="14.25">
       <c r="B220" t="s">
         <v>522</v>
       </c>
@@ -5560,7 +5695,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="221" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="221" spans="2:5" ht="14.25">
       <c r="B221" t="s">
         <v>524</v>
       </c>
@@ -5574,7 +5709,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="222" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="222" spans="2:5" ht="14.25">
       <c r="B222" t="s">
         <v>526</v>
       </c>
@@ -5588,7 +5723,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="223" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="223" spans="2:5" ht="14.25">
       <c r="B223" t="s">
         <v>528</v>
       </c>
@@ -5602,7 +5737,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="224" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="224" spans="2:5" ht="14.25">
       <c r="B224" t="s">
         <v>530</v>
       </c>
@@ -5616,7 +5751,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="225" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="225" spans="2:5" ht="14.25">
       <c r="B225" t="s">
         <v>532</v>
       </c>
@@ -5630,7 +5765,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="226" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="226" spans="2:5" ht="14.25">
       <c r="B226" t="s">
         <v>534</v>
       </c>
@@ -5644,7 +5779,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="227" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="227" spans="2:5" ht="14.25">
       <c r="B227" t="s">
         <v>536</v>
       </c>
@@ -5658,7 +5793,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="228" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="228" spans="2:5" ht="14.25">
       <c r="B228" t="s">
         <v>538</v>
       </c>
@@ -5672,7 +5807,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="229" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="229" spans="2:5" ht="14.25">
       <c r="B229" t="s">
         <v>540</v>
       </c>
@@ -5686,7 +5821,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="230" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="230" spans="2:5" ht="14.25">
       <c r="B230" t="s">
         <v>542</v>
       </c>
@@ -5700,7 +5835,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="231" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="231" spans="2:5" ht="14.25">
       <c r="B231" t="s">
         <v>544</v>
       </c>
@@ -5714,7 +5849,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="232" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="232" spans="2:5" ht="14.25">
       <c r="B232" t="s">
         <v>546</v>
       </c>
@@ -5728,7 +5863,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="233" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="233" spans="2:5" ht="14.25">
       <c r="B233" t="s">
         <v>548</v>
       </c>
@@ -5742,7 +5877,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="234" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="234" spans="2:5" ht="14.25">
       <c r="B234" t="s">
         <v>550</v>
       </c>
@@ -5756,7 +5891,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="235" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="235" spans="2:5" ht="14.25">
       <c r="B235" t="s">
         <v>552</v>
       </c>
@@ -5770,7 +5905,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="236" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="236" spans="2:5" ht="14.25">
       <c r="B236" t="s">
         <v>554</v>
       </c>
@@ -5784,7 +5919,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="237" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="237" spans="2:5" ht="14.25">
       <c r="B237" t="s">
         <v>556</v>
       </c>
@@ -5798,7 +5933,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="238" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="238" spans="2:5" ht="14.25">
       <c r="B238" t="s">
         <v>558</v>
       </c>
@@ -5812,7 +5947,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="239" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="239" spans="2:5" ht="14.25">
       <c r="B239" t="s">
         <v>560</v>
       </c>
@@ -5826,7 +5961,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="240" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="240" spans="2:5" ht="14.25">
       <c r="B240" t="s">
         <v>562</v>
       </c>
@@ -5840,7 +5975,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="241" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="241" spans="2:5" ht="14.25">
       <c r="B241" t="s">
         <v>564</v>
       </c>
@@ -5854,7 +5989,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="242" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="242" spans="2:5" ht="14.25">
       <c r="B242" t="s">
         <v>566</v>
       </c>
@@ -5868,7 +6003,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="243" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="243" spans="2:5" ht="14.25">
       <c r="B243" t="s">
         <v>568</v>
       </c>
@@ -5882,7 +6017,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="244" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="244" spans="2:5" ht="14.25">
       <c r="B244" t="s">
         <v>570</v>
       </c>
@@ -5896,7 +6031,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="245" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="245" spans="2:5" ht="14.25">
       <c r="B245" t="s">
         <v>572</v>
       </c>
@@ -5916,23 +6051,23 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
   <dimension ref="A1:K48"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.86328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.4285714285714" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.4285714285714" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:1" ht="17.25" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:10" ht="15" thickTop="1" thickBot="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -5964,7 +6099,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:9" ht="14.25">
       <c r="B3" t="s">
         <v>91</v>
       </c>
@@ -5981,7 +6116,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:6" ht="14.25">
       <c r="B4" t="s">
         <v>92</v>
       </c>
@@ -5989,7 +6124,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:6" ht="14.25">
       <c r="B5" t="s">
         <v>93</v>
       </c>
@@ -5997,7 +6132,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:9" ht="14.25">
       <c r="B6" t="s">
         <v>94</v>
       </c>
@@ -6011,7 +6146,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:6" ht="14.25">
       <c r="B7" t="s">
         <v>95</v>
       </c>
@@ -6019,7 +6154,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:6" ht="14.25">
       <c r="B8" t="s">
         <v>96</v>
       </c>
@@ -6027,7 +6162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:6" ht="14.25">
       <c r="B9" t="s">
         <v>26</v>
       </c>
@@ -6035,7 +6170,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:6" ht="14.25">
       <c r="B10" t="s">
         <v>97</v>
       </c>
@@ -6043,7 +6178,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="4:6" ht="14.25">
       <c r="D11" t="s">
         <v>33</v>
       </c>
@@ -6051,7 +6186,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:7" ht="14.25">
       <c r="B12" s="3"/>
       <c r="D12" t="s">
         <v>84</v>
@@ -6063,7 +6198,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="4:7" ht="14.25">
       <c r="D13" t="s">
         <v>85</v>
       </c>
@@ -6074,7 +6209,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="4:6" ht="14.25">
       <c r="D14" t="s">
         <v>34</v>
       </c>
@@ -6082,7 +6217,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" ht="14.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -6096,7 +6231,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6" ht="14.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -6110,7 +6245,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:9" ht="14.25">
       <c r="B17" s="3" t="s">
         <v>72</v>
       </c>
@@ -6127,7 +6262,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:6" ht="14.25">
       <c r="B18" t="s">
         <v>70</v>
       </c>
@@ -6138,7 +6273,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:6" ht="14.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -6149,7 +6284,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:9" ht="14.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -6166,7 +6301,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" ht="14.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -6177,7 +6312,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" ht="14.25">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -6188,7 +6323,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" ht="14.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -6196,7 +6331,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:6" ht="14.25">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -6207,7 +6342,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:6" ht="14.25">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -6218,7 +6353,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:11" ht="14.25">
       <c r="B26" t="str">
         <f>"g[_]*"&amp;K26</f>
         <v>g[_]*220</v>
@@ -6231,20 +6366,20 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:11" ht="14.25">
       <c r="B27" t="str">
-        <f t="shared" ref="B27:B46" si="0">"g[_]*"&amp;K27</f>
+        <f t="shared" si="0" ref="B27:B46">"g[_]*"&amp;K27</f>
         <v>g[_]*400</v>
       </c>
       <c r="F27" t="str">
-        <f t="shared" ref="F27:F46" si="1">"Grid-"&amp;K27&amp;"V"</f>
+        <f t="shared" si="1" ref="F27:F46">"Grid-"&amp;K27&amp;"V"</f>
         <v>Grid-400V</v>
       </c>
       <c r="K27">
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:11" ht="14.25">
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*380</v>
@@ -6257,7 +6392,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:11" ht="14.25">
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*225</v>
@@ -6270,7 +6405,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:11" ht="14.25">
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*330</v>
@@ -6283,7 +6418,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:11" ht="14.25">
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*275</v>
@@ -6296,7 +6431,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:11" ht="14.25">
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*420</v>
@@ -6309,7 +6444,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:11" ht="14.25">
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*300</v>
@@ -6322,7 +6457,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:11" ht="14.25">
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*500</v>
@@ -6335,7 +6470,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:11" ht="14.25">
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*750</v>
@@ -6348,7 +6483,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:11" ht="14.25">
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*450</v>
@@ -6361,7 +6496,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:11" ht="14.25">
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*515</v>
@@ -6374,7 +6509,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:11" ht="14.25">
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*525</v>
@@ -6387,7 +6522,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:11" ht="14.25">
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*320</v>
@@ -6400,7 +6535,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:11" ht="14.25">
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*150</v>
@@ -6413,7 +6548,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:11" ht="14.25">
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*270</v>
@@ -6426,7 +6561,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:11" ht="14.25">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*350</v>
@@ -6439,7 +6574,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:11" ht="14.25">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*250</v>
@@ -6452,7 +6587,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:11" ht="14.25">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*200</v>
@@ -6465,7 +6600,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:11" ht="14.25">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*236</v>
@@ -6478,7 +6613,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:11" ht="14.25">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*600</v>
@@ -6491,7 +6626,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:6" ht="14.25">
       <c r="B47" t="s">
         <v>90</v>
       </c>
@@ -6499,7 +6634,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:6" ht="14.25">
       <c r="B48" t="s">
         <v>79</v>
       </c>
@@ -6510,4 +6645,83 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{a8bf2354-7268-48ee-b28f-8d29a8c0893f}">
+  <dimension ref="B2:M4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="2:2" ht="15">
+      <c r="B2" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" ht="15">
+      <c r="B3" t="s">
+        <v>575</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
+        <v>576</v>
+      </c>
+      <c r="E3" t="s">
+        <v>577</v>
+      </c>
+      <c r="F3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G3" t="s">
+        <v>578</v>
+      </c>
+      <c r="H3" t="s">
+        <v>579</v>
+      </c>
+      <c r="I3" t="s">
+        <v>580</v>
+      </c>
+      <c r="J3" t="s">
+        <v>581</v>
+      </c>
+      <c r="K3" t="s">
+        <v>100</v>
+      </c>
+      <c r="L3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="15">
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
+        <v>582</v>
+      </c>
+      <c r="G4" t="s">
+        <v>583</v>
+      </c>
+      <c r="I4" t="s">
+        <v>584</v>
+      </c>
+      <c r="K4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" t="s">
+        <v>585</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>